<commit_message>
Update AI Audit Log_MacTuHau.xlsx
</commit_message>
<xml_diff>
--- a/AI Audit Log_MacTuHau.xlsx
+++ b/AI Audit Log_MacTuHau.xlsx
@@ -5,17 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\GitHub\ai-audit-log-mactuhau\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5392AB06-AB39-4A73-9772-F26E38E421B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94B52E7D-D0BC-4F8C-8FFF-0F6D82DD5FAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{84C35D15-8A6C-4EDA-8B49-2CCD89DED56E}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 1" sheetId="2" r:id="rId1"/>
     <sheet name="Week 2" sheetId="1" r:id="rId2"/>
-    <sheet name="Assignment 3" sheetId="4" r:id="rId3"/>
+    <sheet name="Week 3" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="62">
   <si>
     <t>Giai đoạn/Thành phần DTC</t>
   </si>
@@ -174,6 +174,78 @@
   <si>
     <t>Phản hồi: AI phân biệt rõ sự khác nhau giữa Local Database và Cloud Database. Đồng thời gợi ý dùng gói Azure for Students để tạo server chung hoặc dùng phần mềm Ngrok để mở port máy cá nhân.
 Kiểm chứng &amp; Quyết định: AI không biết rằng tài khoản Azure Student của tôi đang bị lỗi xác thực thẻ (Unable to complete verification). Hơn nữa, việc dùng Ngrok đòi hỏi tôi phải bật máy tính 24/24. Dựa trên tình hình thực tế, tôi đã tự đưa ra giải pháp mới: nhờ một bạn trong nhóm chưa từng dùng Azure dùng email của bạn đó tạo Server, sau đó tôi sẽ đảm nhận việc deploy Database từ máy Local của tôi lên Server đó. Quyết định này giúp nhóm có môi trường làm việc chung 24/7 cực kỳ ổn định mà không tốn chi phí hay phải treo máy liên tục.</t>
+  </si>
+  <si>
+    <t>"Implement the Login page from Figma node 6-2, following 20 architecture rules (feature-based, Zustand, React Query, Zod…)"</t>
+  </si>
+  <si>
+    <t>AI split features/auth/ into api/, services/, hooks/, stores/, validations/, components/, pages/; reusable UI into shared/components/ (InputField, Checkbox, Divider). Decision: Accepted the structure; enforced all API calls through authApi → authService → React Query hooks — never directly in UI. Build passed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	
+Pattern Recognition / Evaluation</t>
+  </si>
+  <si>
+    <t>"Migrate auth from Redux to Zustand; update useAuth, axiosInstance, ProfileMenu"</t>
+  </si>
+  <si>
+    <t>AI created shared/stores/authStore.ts (global session) and loginStore.ts (UI: rememberMe, showPassword). Decision: Separated global vs feature stores (rule 13); migrated auth only, did not remove Redux project-wide to avoid breaking other modules.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	
+Problem Solving</t>
+  </si>
+  <si>
+    <t>"Implement Register from Figma node 6-107, reusing the Login pattern"</t>
+  </si>
+  <si>
+    <t>AI refactored AuthBrandPanel with titleLines prop, added registerSchema, useRegister, registerStore. Decision: Reused login.css for split layout; used Zod .refine() for confirmPassword matching.</t>
+  </si>
+  <si>
+    <t>"Implement the 5-screen Forgot Password flow (Figma 6-216 → 6-532)"</t>
+  </si>
+  <si>
+    <t>AI designed multi-step flow: forgotPasswordStore (method, contact, cooldown, isOtpVerified) + forgotPasswordSuccessStore. Decision: Route chain /forgot-password → /verify → /otp → /reset → /success; guard redirects when state is missing.</t>
+  </si>
+  <si>
+    <t>"Create reusable components for OTP input and method selection cards"</t>
+  </si>
+  <si>
+    <t>AI placed SelectionCard, OtpInput, SuccessIcon, SuccessState in shared/components/. Decision: Generic UI in shared; auth-specific copy/layout in feature. OtpInput supports paste, auto-focus, and keyboard navigation.</t>
+  </si>
+  <si>
+    <t>"Figma MCP quota exhausted — implement OTP / Reset / Success screens"</t>
+  </si>
+  <si>
+    <t>AI could not read nodes 6-382, 6-459, 6-532; inferred layout from prior screens (32px title, primary button + arrow, support footer). Decision: Implemented using existing patterns; pixel-perfect review needed when MCP quota is available. npm run build passed.</t>
+  </si>
+  <si>
+    <t>"Merge main into hau — ProfileMenu.jsx conflict (3 conflicts)"</t>
+  </si>
+  <si>
+    <t>main used Redux dispatch(logout()); hau used Zustand clearAuthSession() + navigate('/login'). Decision: Kept the hau version since auth was already migrated; rejected Redux revert. Merge completed successfully.</t>
+  </si>
+  <si>
+    <t>Evaluation</t>
+  </si>
+  <si>
+    <t>"Handle backend API not yet available"</t>
+  </si>
+  <si>
+    <t>AI added demo fallback: Promise.race with 3s timeout → mock response for login/register/forgot-password. Decision: Accepted for dev/demo; replace with real error handling when BE is deployed.</t>
+  </si>
+  <si>
+    <t>"Validation schemas for each forgot-password step"</t>
+  </si>
+  <si>
+    <t>AI created separate schemas: email/phone verify, 6-digit OTP, reset password + confirm. Decision: One schema per step instead of a monolithic schema; phone regex (0|+84)[0-9]{9,10} for Vietnam.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	
+"Test full flow on dev server"</t>
+  </si>
+  <si>
+    <t>Multiple stale instances occupied ports 5173–5179 → new server on 5180. Decision: Used temporarily; kill old processes before demo. Flow: / → /login → forgot-password → success → /login.</t>
   </si>
 </sst>
 </file>
@@ -924,9 +996,171 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{323516A4-AE23-41CF-AD84-97A6064FC5FB}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="21" customWidth="1"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="24.28515625" customWidth="1"/>
+    <col min="4" max="4" width="76.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="5" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="4"/>
+    </row>
+    <row r="2" spans="1:5" ht="90" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>